<commit_message>
Updated asset naming conventions
</commit_message>
<xml_diff>
--- a/docs/asset-management/PromptCraft_Production_Overview_Simplified.xlsx
+++ b/docs/asset-management/PromptCraft_Production_Overview_Simplified.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rfe4b3ce0c2634e42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Guide" sheetId="2" r:id="R348e6c9447554734"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R8cd7473f7af04475"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Guide" sheetId="2" r:id="R0bba44f762374c96"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -41,6 +41,10 @@
       <x:color rgb="FF203449"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
   <x:fills count="3">
     <x:fill>
@@ -61,7 +65,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="8">
+  <x:cellXfs count="10">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -74,6 +78,10 @@
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -96,8 +104,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ProductionFileGuide" displayName="ProductionFileGuide" ref="A5:B10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:B10"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ProductionFileGuide" displayName="ProductionFileGuide" ref="A5:B11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:B11"/>
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="File"/>
     <x:tableColumn id="2" name="Use it for"/>
@@ -312,11 +320,26 @@
       <x:c r="A2" s="1" t="str">
         <x:v>PromptCraft production work</x:v>
       </x:c>
+      <x:c r="B2"/>
+      <x:c r="C2"/>
+      <x:c r="D2"/>
+      <x:c r="E2"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="2" t="str">
         <x:v>Start with Scenario 1. Work down this list; detailed paths and status fields are in the named workbooks.</x:v>
       </x:c>
+      <x:c r="B3"/>
+      <x:c r="C3"/>
+      <x:c r="D3"/>
+      <x:c r="E3"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4"/>
+      <x:c r="B4"/>
+      <x:c r="C4"/>
+      <x:c r="D4"/>
+      <x:c r="E4"/>
     </x:row>
     <x:row r="5" ht="27" customHeight="1">
       <x:c r="A5" s="5" t="str">
@@ -346,7 +369,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="D6" s="7" t="str">
-        <x:v>Review exact text and proposed filenames</x:v>
+        <x:v>Review exact text and standard filenames</x:v>
       </x:c>
       <x:c r="E6" s="7" t="str">
         <x:v>PromptCraft_Voice_Recording_Tracker.xlsx &gt; S1 Record</x:v>
@@ -423,7 +446,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ac1df31599c4432"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0498524268254290"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -440,11 +463,17 @@
       <x:c r="A2" s="1" t="str">
         <x:v>Which file to open</x:v>
       </x:c>
+      <x:c r="B2"/>
     </x:row>
     <x:row r="3" ht="22" customHeight="1">
       <x:c r="A3" s="2" t="str">
         <x:v>Each workbook has one primary job.</x:v>
       </x:c>
+      <x:c r="B3"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4"/>
+      <x:c r="B4"/>
     </x:row>
     <x:row r="5" ht="27" customHeight="1">
       <x:c r="A5" s="5" t="str">
@@ -494,10 +523,18 @@
         <x:v>Read the current S1 artwork explanation</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="9" t="str">
+        <x:v>ASSET_NAMING_STANDARD.md</x:v>
+      </x:c>
+      <x:c r="B11" s="9" t="str">
+        <x:v>Use the approved audio and visual filename patterns</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e43346b530a4ae9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5769e1721b8d4cde"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed formatting and App Script
</commit_message>
<xml_diff>
--- a/docs/asset-management/PromptCraft_Production_Overview_Simplified.xlsx
+++ b/docs/asset-management/PromptCraft_Production_Overview_Simplified.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R8cd7473f7af04475"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Guide" sheetId="2" r:id="R0bba44f762374c96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R7ac918d8daed4db4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File Guide" sheetId="2" r:id="Re6b5ed2a3fb14913"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,21 +14,33 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="6">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
-      <x:sz val="15"/>
-      <x:color rgb="FF152A42"/>
-      <x:name val="Aptos Display"/>
-    </x:font>
-    <x:font>
+      <x:sz val="16"/>
+      <x:color rgb="FF17324D"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
       <x:sz val="10"/>
-      <x:color rgb="FF526577"/>
-      <x:name val="Aptos"/>
+      <x:color rgb="FF536B7F"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF17324D"/>
+      <x:name val="Arial"/>
     </x:font>
     <x:font>
       <x:b/>
@@ -38,15 +50,23 @@
     </x:font>
     <x:font>
       <x:sz val="10"/>
-      <x:color rgb="FF203449"/>
+      <x:color rgb="FF000000"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
+      <x:b/>
+      <x:sz val="18"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:i/>
       <x:sz val="10"/>
-      <x:name val="Arial"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -55,32 +75,231 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FF183B5D"/>
+        <x:fgColor rgb="FF163F63"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF12355B"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="1">
+  <x:borders count="9">
     <x:border/>
+    <x:border>
+      <x:bottom style="medium">
+        <x:color rgb="FFF2B827"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFFFFFFF"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFFFFFFF"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFFFFFFF"/>
+      </x:right>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFFFFFFF"/>
+      </x:left>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFC8DCE8"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFC8DCE8"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFC8DCE8"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFC8DCE8"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD9D9D9"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="10">
+  <x:cellXfs count="61">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -90,8 +309,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ProductionNextActions" displayName="ProductionNextActions" ref="A5:E10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:E10"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ProductionOrder" displayName="ProductionOrder" ref="A5:E10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="5">
     <x:tableColumn id="1" name="Order"/>
     <x:tableColumn id="2" name="Work"/>
@@ -104,8 +322,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ProductionFileGuide" displayName="ProductionFileGuide" ref="A5:B11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:B11"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="ProductionFileGuide" displayName="ProductionFileGuide" ref="A5:B12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="File"/>
     <x:tableColumn id="2" name="Use it for"/>
@@ -309,144 +526,155 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="35" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="11" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="59" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="72" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="31" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="49" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="54" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="2" ht="27" customHeight="1">
-      <x:c r="A2" s="1" t="str">
+    <x:row r="1">
+      <x:c r="A1" s="55"/>
+      <x:c r="B1" s="55"/>
+      <x:c r="C1" s="55"/>
+      <x:c r="D1" s="55"/>
+      <x:c r="E1" s="55"/>
+    </x:row>
+    <x:row r="2" ht="28" customHeight="1">
+      <x:c r="A2" s="59" t="str">
         <x:v>PromptCraft production work</x:v>
       </x:c>
-      <x:c r="B2"/>
-      <x:c r="C2"/>
-      <x:c r="D2"/>
-      <x:c r="E2"/>
-    </x:row>
-    <x:row r="3" ht="22" customHeight="1">
-      <x:c r="A3" s="2" t="str">
-        <x:v>Start with Scenario 1. Work down this list; detailed paths and status fields are in the named workbooks.</x:v>
-      </x:c>
-      <x:c r="B3"/>
-      <x:c r="C3"/>
-      <x:c r="D3"/>
-      <x:c r="E3"/>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4"/>
-      <x:c r="B4"/>
-      <x:c r="C4"/>
-      <x:c r="D4"/>
-      <x:c r="E4"/>
-    </x:row>
-    <x:row r="5" ht="27" customHeight="1">
-      <x:c r="A5" s="5" t="str">
+      <x:c r="B2" s="59"/>
+      <x:c r="C2" s="59"/>
+      <x:c r="D2" s="59"/>
+      <x:c r="E2" s="59"/>
+    </x:row>
+    <x:row r="3" ht="32" customHeight="1">
+      <x:c r="A3" s="60" t="str">
+        <x:v>Everything below is planned and not started. Begin with wording approval, then use the exact filenames and visual specifications.</x:v>
+      </x:c>
+      <x:c r="B3" s="60"/>
+      <x:c r="C3" s="60"/>
+      <x:c r="D3" s="60"/>
+      <x:c r="E3" s="60"/>
+    </x:row>
+    <x:row r="4" ht="6" customHeight="1">
+      <x:c r="A4" s="58"/>
+      <x:c r="B4" s="58"/>
+      <x:c r="C4" s="58"/>
+      <x:c r="D4" s="58"/>
+      <x:c r="E4" s="58"/>
+    </x:row>
+    <x:row r="5" ht="38" customHeight="1">
+      <x:c r="A5" s="37" t="str">
         <x:v>Order</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="str">
+      <x:c r="B5" s="37" t="str">
         <x:v>Work</x:v>
       </x:c>
-      <x:c r="C5" s="5" t="str">
+      <x:c r="C5" s="37" t="str">
         <x:v>Items</x:v>
       </x:c>
-      <x:c r="D5" s="5" t="str">
+      <x:c r="D5" s="37" t="str">
         <x:v>Next action</x:v>
       </x:c>
-      <x:c r="E5" s="5" t="str">
+      <x:c r="E5" s="37" t="str">
         <x:v>Open</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="27" customHeight="1">
-      <x:c r="A6" s="7" t="n">
+    <x:row r="6" ht="36" customHeight="1">
+      <x:c r="A6" s="53" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="str">
+      <x:c r="B6" s="54" t="str">
         <x:v>Approve S1 spoken lines</x:v>
       </x:c>
-      <x:c r="C6" s="7" t="n">
+      <x:c r="C6" s="53" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="D6" s="7" t="str">
-        <x:v>Review exact text and standard filenames</x:v>
-      </x:c>
-      <x:c r="E6" s="7" t="str">
+      <x:c r="D6" s="54" t="str">
+        <x:v>Review the exact wording, source IDs, and planned filenames</x:v>
+      </x:c>
+      <x:c r="E6" s="54" t="str">
         <x:v>PromptCraft_Voice_Recording_Tracker.xlsx &gt; S1 Record</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="27" customHeight="1">
-      <x:c r="A7" s="7" t="n">
+    <x:row r="7" ht="36" customHeight="1">
+      <x:c r="A7" s="53" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B7" s="7" t="str">
+      <x:c r="B7" s="54" t="str">
         <x:v>Record and check audio</x:v>
       </x:c>
-      <x:c r="C7" s="7" t="n">
+      <x:c r="C7" s="53" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="D7" s="7" t="str">
+      <x:c r="D7" s="54" t="str">
         <x:v>After approval, record one file per line</x:v>
       </x:c>
-      <x:c r="E7" s="7" t="str">
+      <x:c r="E7" s="54" t="str">
         <x:v>PromptCraft_Voice_Recording_Tracker.xlsx &gt; S1 Record</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="27" customHeight="1">
-      <x:c r="A8" s="7" t="n">
+    <x:row r="8" ht="36" customHeight="1">
+      <x:c r="A8" s="53" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B8" s="7" t="str">
-        <x:v>Check current S1 artwork</x:v>
-      </x:c>
-      <x:c r="C8" s="7" t="n">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="D8" s="7" t="str">
-        <x:v>Review phone, tablet, Nest Hub, and desktop framing</x:v>
-      </x:c>
-      <x:c r="E8" s="7" t="str">
-        <x:v>PromptCraft_Visual_Asset_Tracker_Simplified.xlsx &gt; S1 Artwork</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="27" customHeight="1">
-      <x:c r="A9" s="7" t="n">
+      <x:c r="B8" s="54" t="str">
+        <x:v>Decide optional Maya voices</x:v>
+      </x:c>
+      <x:c r="C8" s="53" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D8" s="54" t="str">
+        <x:v>Review every fixed and conditional Maya line before recording extras</x:v>
+      </x:c>
+      <x:c r="E8" s="54" t="str">
+        <x:v>S1_Maya_Recording_Script.docx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="36" customHeight="1">
+      <x:c r="A9" s="53" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B9" s="7" t="str">
-        <x:v>Decide whether to voice on screen quotes</x:v>
-      </x:c>
-      <x:c r="C9" s="7" t="n">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="D9" s="7" t="str">
-        <x:v>Keep unapproved quotes out of the audio queue</x:v>
-      </x:c>
-      <x:c r="E9" s="7" t="str">
-        <x:v>PromptCraft_Voice_Recording_Tracker.xlsx &gt; S1 On Screen</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="27" customHeight="1">
-      <x:c r="A10" s="7" t="n">
+      <x:c r="B9" s="54" t="str">
+        <x:v>Create required S1 artwork</x:v>
+      </x:c>
+      <x:c r="C9" s="53" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="D9" s="54" t="str">
+        <x:v>Use exact dimensions, paths, and code keys</x:v>
+      </x:c>
+      <x:c r="E9" s="54" t="str">
+        <x:v>S1_Asset_Production_Specifications.docx</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="36" customHeight="1">
+      <x:c r="A10" s="53" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B10" s="7" t="str">
-        <x:v>Review older Canvas art later</x:v>
-      </x:c>
-      <x:c r="C10" s="7" t="n">
-        <x:v>25</x:v>
-      </x:c>
-      <x:c r="D10" s="7" t="str">
-        <x:v>Check 24 registered captures and 1 reference before lifecycle changes</x:v>
-      </x:c>
-      <x:c r="E10" s="7" t="str">
-        <x:v>PromptCraft_Visual_Asset_Tracker_Simplified.xlsx &gt; Legacy S1</x:v>
+      <x:c r="B10" s="54" t="str">
+        <x:v>Review choices and feedback</x:v>
+      </x:c>
+      <x:c r="C10" s="53" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="D10" s="54" t="str">
+        <x:v>Review choices, validation, fallback, and dynamic templates</x:v>
+      </x:c>
+      <x:c r="E10" s="54" t="str">
+        <x:v>PromptCraft_Voice_Recording_Tracker.xlsx &gt; S1 Choices &amp; Feedback</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:E2"/>
+    <x:mergeCell ref="A3:E3"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0498524268254290"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa6997931c3a46e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -455,86 +683,98 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="64" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="75" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="52" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="84" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="2" ht="27" customHeight="1">
-      <x:c r="A2" s="1" t="str">
+    <x:row r="1">
+      <x:c r="A1" s="55"/>
+      <x:c r="B1" s="55"/>
+    </x:row>
+    <x:row r="2" ht="21" customHeight="1">
+      <x:c r="A2" s="56" t="str">
         <x:v>Which file to open</x:v>
       </x:c>
-      <x:c r="B2"/>
-    </x:row>
-    <x:row r="3" ht="22" customHeight="1">
-      <x:c r="A3" s="2" t="str">
-        <x:v>Each workbook has one primary job.</x:v>
-      </x:c>
-      <x:c r="B3"/>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4"/>
-      <x:c r="B4"/>
-    </x:row>
-    <x:row r="5" ht="27" customHeight="1">
-      <x:c r="A5" s="5" t="str">
+      <x:c r="B2" s="56"/>
+    </x:row>
+    <x:row r="3" ht="18" customHeight="1">
+      <x:c r="A3" s="57" t="str">
+        <x:v>Each document has one production job.</x:v>
+      </x:c>
+      <x:c r="B3" s="57"/>
+    </x:row>
+    <x:row r="4" ht="6" customHeight="1">
+      <x:c r="A4" s="58"/>
+      <x:c r="B4" s="58"/>
+    </x:row>
+    <x:row r="5" ht="38" customHeight="1">
+      <x:c r="A5" s="37" t="str">
         <x:v>File</x:v>
       </x:c>
-      <x:c r="B5" s="5" t="str">
+      <x:c r="B5" s="37" t="str">
         <x:v>Use it for</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="27" customHeight="1">
-      <x:c r="A6" s="7" t="str">
+    <x:row r="6" ht="28.5" customHeight="1">
+      <x:c r="A6" s="54" t="str">
         <x:v>PromptCraft_Voice_Recording_Tracker.xlsx</x:v>
       </x:c>
-      <x:c r="B6" s="7" t="str">
-        <x:v>Approve, record, and check S1 lines; keep other audio separate</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="27" customHeight="1">
-      <x:c r="A7" s="7" t="str">
+      <x:c r="B6" s="54" t="str">
+        <x:v>Approve nine spoken lines, reserve optional Maya filenames, and review all fixed branch text</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="28.5" customHeight="1">
+      <x:c r="A7" s="54" t="str">
         <x:v>PromptCraft_Visual_Asset_Tracker_Simplified.xlsx</x:v>
       </x:c>
-      <x:c r="B7" s="7" t="str">
-        <x:v>Check current S1 art and look up all artwork paths</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="27" customHeight="1">
-      <x:c r="A8" s="7" t="str">
+      <x:c r="B7" s="54" t="str">
+        <x:v>Use exact filenames, dimensions, destination folders, and code references for 12 S1 visuals</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="28.5" customHeight="1">
+      <x:c r="A8" s="54" t="str">
         <x:v>S1_Professor_Pixel_Recording_Script.docx</x:v>
       </x:c>
-      <x:c r="B8" s="7" t="str">
-        <x:v>Read Professor Pixel lines and proposed file paths</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="27" customHeight="1">
-      <x:c r="A9" s="7" t="str">
+      <x:c r="B8" s="54" t="str">
+        <x:v>Record Professor Pixel’s six current S1 lines</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="28.5" customHeight="1">
+      <x:c r="A9" s="54" t="str">
         <x:v>S1_Maya_Recording_Script.docx</x:v>
       </x:c>
-      <x:c r="B9" s="7" t="str">
-        <x:v>Read Maya lines and proposed file paths</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="27" customHeight="1">
-      <x:c r="A10" s="7" t="str">
-        <x:v>S1_ARTWORK_CURRENT.md</x:v>
-      </x:c>
-      <x:c r="B10" s="7" t="str">
-        <x:v>Read the current S1 artwork explanation</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="9" t="str">
+      <x:c r="B9" s="54" t="str">
+        <x:v>Record Maya’s three main lines and review all optional and conditional Maya lines</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="28.5" customHeight="1">
+      <x:c r="A10" s="54" t="str">
+        <x:v>S1_Asset_Production_Specifications.docx</x:v>
+      </x:c>
+      <x:c r="B10" s="54" t="str">
+        <x:v>Use one printable map for artwork dimensions, export formats, folders, and code references</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="28.5" customHeight="1">
+      <x:c r="A11" s="54" t="str">
+        <x:v>S1_ARTWORK_PLAN.md</x:v>
+      </x:c>
+      <x:c r="B11" s="54" t="str">
+        <x:v>Read the concise artwork brief and size guide</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="54" t="str">
         <x:v>ASSET_NAMING_STANDARD.md</x:v>
       </x:c>
-      <x:c r="B11" s="9" t="str">
+      <x:c r="B12" s="54" t="str">
         <x:v>Use the approved audio and visual filename patterns</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5769e1721b8d4cde"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red2ee10f018f436e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>